<commit_message>
changes, mainly excel files for pricing data and with the button to add new excel files
</commit_message>
<xml_diff>
--- a/data/reference/classification_validation/broker_classification_validation.xlsx
+++ b/data/reference/classification_validation/broker_classification_validation.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sunocoinc-my.sharepoint.com/personal/aftikhar_mominzada_sunoco_com/Documents/Documents/Projects/Index_App/Index_App/data/reference/classification_validation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sunocoinc-my.sharepoint.com/personal/aftikhar_mominzada_sunoco_com/Documents/Documents/Index_App/data/reference/classification_validation/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="169" documentId="13_ncr:20001_{C22BA8CE-55D4-4424-AF1B-3810F59EA028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{892D5A22-5EB0-4C0F-97C9-A12268621AFC}"/>
+  <xr:revisionPtr revIDLastSave="281" documentId="13_ncr:20001_{C22BA8CE-55D4-4424-AF1B-3810F59EA028}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{427ED5AD-FF3C-4C92-A5C1-29E03CC078C8}"/>
   <bookViews>
-    <workbookView xWindow="-63315" yWindow="-11895" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-63315" yWindow="-11895" windowWidth="29040" windowHeight="15720" tabRatio="843" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" r:id="rId1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4366" uniqueCount="1137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4506" uniqueCount="1148">
   <si>
     <t>Item</t>
   </si>
@@ -3457,6 +3457,39 @@
   </si>
   <si>
     <t>SW ICE 1a Index - EDM PEA</t>
+  </si>
+  <si>
+    <t>SYN - EDM ENB</t>
+  </si>
+  <si>
+    <t>PSY - EDM ENB</t>
+  </si>
+  <si>
+    <t>SSP - EDM AOSPL</t>
+  </si>
+  <si>
+    <t>CNS - EDM HZN</t>
+  </si>
+  <si>
+    <t>HSC - HAR ENB</t>
+  </si>
+  <si>
+    <t>SYN - EDM EIL</t>
+  </si>
+  <si>
+    <t>PAS - EDM TMPL</t>
+  </si>
+  <si>
+    <t>PAS</t>
+  </si>
+  <si>
+    <t>SYN_EIL</t>
+  </si>
+  <si>
+    <t>SYN ICE 1A INDEX - EDM ENB</t>
+  </si>
+  <si>
+    <t>SYN Bi4 Index - EDM ENB</t>
   </si>
 </sst>
 </file>
@@ -3466,7 +3499,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3486,6 +3519,13 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="6">
@@ -3518,7 +3558,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -3561,11 +3601,48 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFD9E2F3"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -3594,6 +3671,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3992,7 +4084,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:T251"/>
+  <dimension ref="A1:T256"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -14552,6 +14644,196 @@
       </c>
       <c r="T251" s="3"/>
     </row>
+    <row r="252" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A252" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B252" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C252" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D252" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="K252" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="L252" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M252" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="O252" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="P252" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q252" s="3">
+        <v>100</v>
+      </c>
+      <c r="R252" s="3" t="s">
+        <v>375</v>
+      </c>
+      <c r="S252" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="253" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A253" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B253" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C253" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D253" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="K253" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="L253" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M253" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="O253" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="P253" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="Q253" s="3">
+        <v>100</v>
+      </c>
+      <c r="R253" s="3" t="s">
+        <v>377</v>
+      </c>
+      <c r="S253" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="254" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A254" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B254" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C254" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D254" s="11" t="s">
+        <v>398</v>
+      </c>
+      <c r="K254" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="L254" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M254" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="O254" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="P254" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="Q254" s="3">
+        <v>100</v>
+      </c>
+      <c r="R254" s="3" t="s">
+        <v>379</v>
+      </c>
+      <c r="S254" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="255" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A255" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B255" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C255" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D255" s="11" t="s">
+        <v>413</v>
+      </c>
+      <c r="K255" s="7" t="s">
+        <v>413</v>
+      </c>
+      <c r="L255" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M255" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="O255" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="P255" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q255" s="3">
+        <v>100</v>
+      </c>
+      <c r="R255" s="3" t="s">
+        <v>381</v>
+      </c>
+      <c r="S255" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A256" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="B256" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="C256" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D256" s="11" t="s">
+        <v>415</v>
+      </c>
+      <c r="K256" s="7" t="s">
+        <v>1146</v>
+      </c>
+      <c r="L256" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="M256" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="O256" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="P256" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q256" s="3">
+        <v>100</v>
+      </c>
+      <c r="R256" s="3" t="s">
+        <v>383</v>
+      </c>
+      <c r="S256" s="7" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T251" xr:uid="{00000000-0009-0000-0000-000001000000}">
     <filterColumn colId="12">
@@ -14572,7 +14854,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:T180"/>
+  <dimension ref="A1:T183"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -14585,7 +14867,8 @@
     <col min="12" max="12" width="8" customWidth="1"/>
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="14" width="10" customWidth="1"/>
-    <col min="15" max="16" width="20" customWidth="1"/>
+    <col min="15" max="15" width="20" customWidth="1"/>
+    <col min="16" max="16" width="21.36328125" customWidth="1"/>
     <col min="17" max="17" width="14" customWidth="1"/>
     <col min="18" max="18" width="18" customWidth="1"/>
     <col min="19" max="19" width="10" customWidth="1"/>
@@ -22015,26 +22298,175 @@
       </c>
     </row>
     <row r="180" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A180" s="3"/>
-      <c r="B180" s="3"/>
-      <c r="C180" s="3"/>
-      <c r="D180" s="3"/>
-      <c r="E180" s="3"/>
+      <c r="A180" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B180" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="C180" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D180" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="E180" s="3" t="s">
+        <v>899</v>
+      </c>
       <c r="F180" s="3"/>
       <c r="G180" s="3"/>
       <c r="H180" s="3"/>
       <c r="I180" s="3"/>
       <c r="J180" s="3"/>
-      <c r="K180" s="3"/>
-      <c r="L180" s="3"/>
-      <c r="M180" s="3"/>
+      <c r="K180" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="L180" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M180" s="3" t="s">
+        <v>47</v>
+      </c>
       <c r="N180" s="3"/>
-      <c r="O180" s="3"/>
-      <c r="P180" s="3"/>
-      <c r="Q180" s="3"/>
-      <c r="R180" s="3"/>
-      <c r="S180" s="3"/>
+      <c r="O180" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="P180" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q180" s="3">
+        <v>100</v>
+      </c>
+      <c r="R180" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="S180" s="3" t="b">
+        <v>1</v>
+      </c>
       <c r="T180" s="3"/>
+    </row>
+    <row r="181" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A181" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B181" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="C181" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D181" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="E181" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="K181" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="L181" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M181" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="O181" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="P181" s="7" t="s">
+        <v>398</v>
+      </c>
+      <c r="Q181" s="3">
+        <v>100</v>
+      </c>
+      <c r="R181" s="3" t="s">
+        <v>813</v>
+      </c>
+      <c r="S181" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A182" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B182" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="C182" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D182" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="E182" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="K182" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="L182" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M182" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="O182" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="P182" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="Q182" s="3">
+        <v>100</v>
+      </c>
+      <c r="R182" s="3" t="s">
+        <v>815</v>
+      </c>
+      <c r="S182" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A183" s="3" t="s">
+        <v>556</v>
+      </c>
+      <c r="B183" s="3" t="s">
+        <v>557</v>
+      </c>
+      <c r="C183" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D183" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="E183" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="K183" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="L183" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M183" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="O183" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="P183" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="Q183" s="3">
+        <v>100</v>
+      </c>
+      <c r="R183" s="3" t="s">
+        <v>817</v>
+      </c>
+      <c r="S183" s="3" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:T180" xr:uid="{00000000-0009-0000-0000-000002000000}">
@@ -22052,7 +22484,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:T103"/>
+  <dimension ref="A1:T104"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -26261,6 +26693,44 @@
         <v>328</v>
       </c>
     </row>
+    <row r="104" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A104" s="3" t="s">
+        <v>900</v>
+      </c>
+      <c r="B104" s="3" t="s">
+        <v>901</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D104" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="E104" s="3" t="s">
+        <v>899</v>
+      </c>
+      <c r="K104" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="M104" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="O104" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="P104" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="Q104" s="3">
+        <v>100</v>
+      </c>
+      <c r="R104" s="3" t="s">
+        <v>1056</v>
+      </c>
+      <c r="S104" s="3" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:T103" xr:uid="{00000000-0009-0000-0000-000003000000}">
     <filterColumn colId="12">
@@ -26280,7 +26750,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:T22"/>
+  <dimension ref="A1:T31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -26719,20 +27189,173 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="4:19" x14ac:dyDescent="0.35">
-      <c r="D22" t="s">
+    <row r="22" spans="4:19" s="14" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D22" s="14" t="s">
         <v>1129</v>
       </c>
-      <c r="M22" t="s">
+      <c r="M22" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="O22" t="s">
+      <c r="O22" s="14" t="s">
         <v>230</v>
       </c>
-      <c r="P22" t="s">
+      <c r="P22" s="14" t="s">
         <v>358</v>
       </c>
-      <c r="S22" s="3" t="b">
+      <c r="S22" s="15" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="4:19" s="10" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="D23" s="10" t="s">
+        <v>1137</v>
+      </c>
+      <c r="M23" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O23" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P23" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="S23" s="13" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="4:19" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D24" s="10" t="s">
+        <v>1138</v>
+      </c>
+      <c r="M24" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O24" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="P24" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="S24" s="12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="4:19" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D25" s="10" t="s">
+        <v>1139</v>
+      </c>
+      <c r="M25" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O25" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P25" s="10" t="s">
+        <v>398</v>
+      </c>
+      <c r="S25" s="12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="4:19" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D26" s="10" t="s">
+        <v>1140</v>
+      </c>
+      <c r="M26" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O26" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P26" s="10" t="s">
+        <v>214</v>
+      </c>
+      <c r="S26" s="12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="4:19" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D27" s="10" t="s">
+        <v>1141</v>
+      </c>
+      <c r="M27" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O27" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P27" s="10" t="s">
+        <v>708</v>
+      </c>
+      <c r="S27" s="12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="4:19" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D28" s="10" t="s">
+        <v>1142</v>
+      </c>
+      <c r="M28" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O28" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P28" s="10" t="s">
+        <v>1145</v>
+      </c>
+      <c r="S28" s="12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="4:19" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D29" s="10" t="s">
+        <v>1143</v>
+      </c>
+      <c r="M29" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="O29" s="10" t="s">
+        <v>368</v>
+      </c>
+      <c r="P29" s="10" t="s">
+        <v>1144</v>
+      </c>
+      <c r="S29" s="12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="4:19" s="10" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="D30" s="16" t="s">
+        <v>1147</v>
+      </c>
+      <c r="M30" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="O30" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P30" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="S30" s="12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="4:19" x14ac:dyDescent="0.35">
+      <c r="D31" s="16" t="s">
+        <v>415</v>
+      </c>
+      <c r="M31" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="O31" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P31" s="10" t="s">
+        <v>215</v>
+      </c>
+      <c r="S31" s="12" t="b">
         <v>1</v>
       </c>
     </row>

</xml_diff>